<commit_message>
Se añadio el reporte de CBO
</commit_message>
<xml_diff>
--- a/Metricas/Reportes/CBO_Reporte.xlsx
+++ b/Metricas/Reportes/CBO_Reporte.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alumnosuady-my.sharepoint.com/personal/a23216399_alumnos_uady_mx/Documents/Métricas de SW/proyecto/Plantillas de reportes/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\EBOGE METRICAS\EBOGE\Metricas\Reportes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_868F3FCD1B10314CEC3A2976BE8E9E0D98DCB24E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{770500F1-38CF-4729-B81D-3A33CD609E01}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{697F2FD9-1BB9-45EB-9787-8907C8A15953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -34,8 +34,60 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="4">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="4">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="64">
   <si>
     <t>Resumen</t>
   </si>
@@ -218,6 +270,15 @@
   </si>
   <si>
     <t>TreeMap CBO</t>
+  </si>
+  <si>
+    <t>Aldrin Novelo</t>
+  </si>
+  <si>
+    <t>CBO mide el número de clases externas a las que una clase hace referencia directa, excluyendo herencia. Es un indicador del esfuerzo requerido para mantener y probar el sistema.</t>
+  </si>
+  <si>
+    <t>Se analizó un total de 32 clases pertenecientes a los módulos centrales del sistema EBOGE. Los resultados indican que la arquitectura mantiene un nivel de acoplamiento altamente controlado, concentrando a la gran mayoría de los componentes, 28 clases (87.5%), en el nivel de riesgo Bajo. En el nivel Bajo-medio se identificaron 3 clases (9.4%): Partida, Mazo y GrilletesDelAlma. Finalmente, solo 1 clase (3.1%) se posicionó en el nivel Medio-alto: MotorDeTurnos con un CBO de 12, siendo la que presenta el valor más alto del sistema. Dado que ninguna clase alcanzó los niveles de riesgo Alto o Muy alto, el diseño no presenta fragilidad estructural por exceso de dependencias.</t>
   </si>
 </sst>
 </file>
@@ -577,7 +638,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -649,10 +710,17 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -660,13 +728,9 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -743,111 +807,83 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="4876800" cy="4705350"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="image2.png" title="Imagen">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="180975" cy="190500"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="image3.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000004000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="314325" cy="190500"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="image4.png">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000005000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1059,18 +1095,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="5:6" ht="14.4">
-      <c r="E1" s="27"/>
-      <c r="F1" s="28"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="30"/>
     </row>
     <row r="2" spans="5:6" ht="33.6">
-      <c r="E2" s="29" t="s">
+      <c r="E2" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="30"/>
+      <c r="F2" s="33"/>
     </row>
     <row r="3" spans="5:6" ht="14.4">
-      <c r="E3" s="27"/>
-      <c r="F3" s="28"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="30"/>
     </row>
     <row r="4" spans="5:6" ht="14.4">
       <c r="E4" s="1"/>
@@ -1112,35 +1148,41 @@
       <c r="E9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="5"/>
+      <c r="F9" s="5" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="10" spans="5:6" ht="14.4">
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="5:6" ht="15.6">
-      <c r="E11" s="31" t="s">
+      <c r="E11" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="28"/>
+      <c r="F11" s="30"/>
     </row>
     <row r="12" spans="5:6" ht="75.75" customHeight="1">
-      <c r="E12" s="32"/>
-      <c r="F12" s="28"/>
+      <c r="E12" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" s="35"/>
     </row>
     <row r="13" spans="5:6" ht="14.4">
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
     <row r="14" spans="5:6" ht="15.6">
-      <c r="E14" s="33" t="s">
+      <c r="E14" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="F14" s="34"/>
-    </row>
-    <row r="15" spans="5:6" ht="72.75" customHeight="1">
-      <c r="E15" s="32"/>
-      <c r="F15" s="28"/>
+      <c r="F14" s="28"/>
+    </row>
+    <row r="15" spans="5:6" ht="131.4" customHeight="1">
+      <c r="E15" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="F15" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1202,7 +1244,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="9" t="str">
-        <f>IF(C4&gt;=30, "Muy-alto", IF(C4&gt;=20, "Alto", IF(C4&gt;=10, "Medio-alto", IF(C4&gt;=5, "Bajo-medio", "Bajo"))))</f>
+        <f>IF(C4&gt;30,"Muy-alto",IF(C4&gt;=21,"Alto",IF(C4&gt;=11,"Medio-alto",IF(C4&gt;=6,"Bajo-medio","Bajo"))))</f>
         <v>Bajo</v>
       </c>
     </row>
@@ -1217,7 +1259,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="9" t="str">
-        <f t="shared" ref="D5:D35" si="0">IF(C5&gt;=30, "Muy alto", IF(C5&gt;=20, "Alto", IF(C5&gt;=10, "Medio-alto", IF(C5&gt;=5, "Bajo-medio", "Bajo"))))</f>
+        <f t="shared" ref="D5:D35" si="0">IF(C5&gt;30,"Muy-alto",IF(C5&gt;=21,"Alto",IF(C5&gt;=11,"Medio-alto",IF(C5&gt;=6,"Bajo-medio","Bajo"))))</f>
         <v>Bajo</v>
       </c>
       <c r="F5" s="11"/>
@@ -1399,7 +1441,7 @@
       </c>
       <c r="D17" s="9" t="str">
         <f t="shared" si="0"/>
-        <v>Medio-alto</v>
+        <v>Bajo-medio</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="14.25" customHeight="1">
@@ -1459,7 +1501,7 @@
       </c>
       <c r="D21" s="9" t="str">
         <f t="shared" si="0"/>
-        <v>Bajo-medio</v>
+        <v>Bajo</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="14.25" customHeight="1">
@@ -1489,7 +1531,7 @@
       </c>
       <c r="D23" s="9" t="str">
         <f t="shared" si="0"/>
-        <v>Bajo-medio</v>
+        <v>Bajo</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="14.25" customHeight="1">
@@ -2676,7 +2718,7 @@
     <col min="5" max="5" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" ht="14.4">
       <c r="A1" s="26"/>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -2684,262 +2726,266 @@
       <c r="E1" s="26"/>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="28"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="30"/>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="34"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="26"/>
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="34"/>
+      <c r="E3" s="28"/>
     </row>
     <row r="4" spans="1:5" ht="14.4">
-      <c r="A4" s="36"/>
-      <c r="B4" s="37"/>
+      <c r="A4" s="37" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="B4" s="38"/>
       <c r="C4" s="26"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="37"/>
+      <c r="D4" s="45" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E4" s="38"/>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1">
-      <c r="A5" s="38"/>
-      <c r="B5" s="39"/>
+      <c r="A5" s="39"/>
+      <c r="B5" s="40"/>
       <c r="C5" s="26"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="39"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="40"/>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1">
-      <c r="A6" s="38"/>
-      <c r="B6" s="39"/>
+      <c r="A6" s="39"/>
+      <c r="B6" s="40"/>
       <c r="C6" s="26"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="39"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="40"/>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1">
-      <c r="A7" s="38"/>
-      <c r="B7" s="39"/>
+      <c r="A7" s="39"/>
+      <c r="B7" s="40"/>
       <c r="C7" s="26"/>
-      <c r="D7" s="38"/>
-      <c r="E7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="40"/>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1">
-      <c r="A8" s="38"/>
-      <c r="B8" s="39"/>
+      <c r="A8" s="39"/>
+      <c r="B8" s="40"/>
       <c r="C8" s="26"/>
-      <c r="D8" s="38"/>
-      <c r="E8" s="39"/>
+      <c r="D8" s="39"/>
+      <c r="E8" s="40"/>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1">
-      <c r="A9" s="38"/>
-      <c r="B9" s="39"/>
+      <c r="A9" s="39"/>
+      <c r="B9" s="40"/>
       <c r="C9" s="26"/>
-      <c r="D9" s="38"/>
-      <c r="E9" s="39"/>
+      <c r="D9" s="39"/>
+      <c r="E9" s="40"/>
     </row>
     <row r="10" spans="1:5" ht="15" customHeight="1">
-      <c r="A10" s="38"/>
-      <c r="B10" s="39"/>
+      <c r="A10" s="39"/>
+      <c r="B10" s="40"/>
       <c r="C10" s="26"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="40"/>
     </row>
     <row r="11" spans="1:5" ht="15" customHeight="1">
-      <c r="A11" s="38"/>
-      <c r="B11" s="39"/>
+      <c r="A11" s="39"/>
+      <c r="B11" s="40"/>
       <c r="C11" s="26"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="40"/>
     </row>
     <row r="12" spans="1:5" ht="15" customHeight="1">
-      <c r="A12" s="38"/>
-      <c r="B12" s="39"/>
+      <c r="A12" s="39"/>
+      <c r="B12" s="40"/>
       <c r="C12" s="26"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="39"/>
+      <c r="D12" s="39"/>
+      <c r="E12" s="40"/>
     </row>
     <row r="13" spans="1:5" ht="15" customHeight="1">
-      <c r="A13" s="38"/>
-      <c r="B13" s="39"/>
+      <c r="A13" s="39"/>
+      <c r="B13" s="40"/>
       <c r="C13" s="26"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="40"/>
     </row>
     <row r="14" spans="1:5" ht="15" customHeight="1">
-      <c r="A14" s="38"/>
-      <c r="B14" s="39"/>
+      <c r="A14" s="39"/>
+      <c r="B14" s="40"/>
       <c r="C14" s="26"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="40"/>
     </row>
     <row r="15" spans="1:5" ht="15" customHeight="1">
-      <c r="A15" s="38"/>
-      <c r="B15" s="39"/>
+      <c r="A15" s="39"/>
+      <c r="B15" s="40"/>
       <c r="C15" s="26"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="39"/>
+      <c r="D15" s="39"/>
+      <c r="E15" s="40"/>
     </row>
     <row r="16" spans="1:5" ht="15" customHeight="1">
-      <c r="A16" s="38"/>
-      <c r="B16" s="39"/>
+      <c r="A16" s="39"/>
+      <c r="B16" s="40"/>
       <c r="C16" s="26"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="40"/>
     </row>
     <row r="17" spans="1:5" ht="15" customHeight="1">
-      <c r="A17" s="38"/>
-      <c r="B17" s="39"/>
+      <c r="A17" s="39"/>
+      <c r="B17" s="40"/>
       <c r="C17" s="26"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="39"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="40"/>
     </row>
     <row r="18" spans="1:5" ht="15" customHeight="1">
-      <c r="A18" s="38"/>
-      <c r="B18" s="39"/>
+      <c r="A18" s="39"/>
+      <c r="B18" s="40"/>
       <c r="C18" s="26"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="39"/>
+      <c r="D18" s="39"/>
+      <c r="E18" s="40"/>
     </row>
     <row r="19" spans="1:5" ht="15" customHeight="1">
-      <c r="A19" s="38"/>
-      <c r="B19" s="39"/>
+      <c r="A19" s="39"/>
+      <c r="B19" s="40"/>
       <c r="C19" s="26"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="39"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="40"/>
     </row>
     <row r="20" spans="1:5" ht="15" customHeight="1">
-      <c r="A20" s="38"/>
-      <c r="B20" s="39"/>
+      <c r="A20" s="39"/>
+      <c r="B20" s="40"/>
       <c r="C20" s="26"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="39"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="40"/>
     </row>
     <row r="21" spans="1:5" ht="15" customHeight="1">
-      <c r="A21" s="38"/>
-      <c r="B21" s="39"/>
+      <c r="A21" s="39"/>
+      <c r="B21" s="40"/>
       <c r="C21" s="26"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="39"/>
+      <c r="D21" s="39"/>
+      <c r="E21" s="40"/>
     </row>
     <row r="22" spans="1:5" ht="15" customHeight="1">
-      <c r="A22" s="38"/>
-      <c r="B22" s="39"/>
+      <c r="A22" s="39"/>
+      <c r="B22" s="40"/>
       <c r="C22" s="26"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="39"/>
+      <c r="D22" s="39"/>
+      <c r="E22" s="40"/>
     </row>
     <row r="23" spans="1:5" ht="15" customHeight="1">
-      <c r="A23" s="38"/>
-      <c r="B23" s="39"/>
+      <c r="A23" s="39"/>
+      <c r="B23" s="40"/>
       <c r="C23" s="26"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="39"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="40"/>
     </row>
     <row r="24" spans="1:5" ht="15" customHeight="1">
-      <c r="A24" s="38"/>
-      <c r="B24" s="39"/>
+      <c r="A24" s="39"/>
+      <c r="B24" s="40"/>
       <c r="C24" s="26"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="39"/>
+      <c r="D24" s="39"/>
+      <c r="E24" s="40"/>
     </row>
     <row r="25" spans="1:5" ht="15" customHeight="1">
-      <c r="A25" s="38"/>
-      <c r="B25" s="39"/>
+      <c r="A25" s="39"/>
+      <c r="B25" s="40"/>
       <c r="C25" s="26"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="39"/>
+      <c r="D25" s="39"/>
+      <c r="E25" s="40"/>
     </row>
     <row r="26" spans="1:5" ht="15" customHeight="1">
-      <c r="A26" s="38"/>
-      <c r="B26" s="39"/>
+      <c r="A26" s="39"/>
+      <c r="B26" s="40"/>
       <c r="C26" s="26"/>
-      <c r="D26" s="38"/>
-      <c r="E26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="40"/>
     </row>
     <row r="27" spans="1:5" ht="15" customHeight="1">
-      <c r="A27" s="38"/>
-      <c r="B27" s="39"/>
+      <c r="A27" s="39"/>
+      <c r="B27" s="40"/>
       <c r="C27" s="26"/>
-      <c r="D27" s="38"/>
-      <c r="E27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="40"/>
     </row>
     <row r="28" spans="1:5" ht="14.4">
-      <c r="A28" s="38"/>
-      <c r="B28" s="39"/>
+      <c r="A28" s="39"/>
+      <c r="B28" s="40"/>
       <c r="C28" s="26"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="39"/>
+      <c r="D28" s="39"/>
+      <c r="E28" s="40"/>
     </row>
     <row r="29" spans="1:5" ht="14.4">
-      <c r="A29" s="38"/>
-      <c r="B29" s="39"/>
+      <c r="A29" s="39"/>
+      <c r="B29" s="40"/>
       <c r="C29" s="26"/>
-      <c r="D29" s="38"/>
-      <c r="E29" s="39"/>
+      <c r="D29" s="39"/>
+      <c r="E29" s="40"/>
     </row>
     <row r="30" spans="1:5" ht="14.4">
-      <c r="A30" s="38"/>
-      <c r="B30" s="39"/>
+      <c r="A30" s="39"/>
+      <c r="B30" s="40"/>
       <c r="C30" s="26"/>
-      <c r="D30" s="38"/>
-      <c r="E30" s="39"/>
+      <c r="D30" s="39"/>
+      <c r="E30" s="40"/>
     </row>
     <row r="31" spans="1:5" ht="14.4">
-      <c r="A31" s="38"/>
-      <c r="B31" s="39"/>
+      <c r="A31" s="39"/>
+      <c r="B31" s="40"/>
       <c r="C31" s="26"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="39"/>
+      <c r="D31" s="39"/>
+      <c r="E31" s="40"/>
     </row>
     <row r="32" spans="1:5" ht="14.4">
-      <c r="A32" s="38"/>
-      <c r="B32" s="39"/>
+      <c r="A32" s="39"/>
+      <c r="B32" s="40"/>
       <c r="C32" s="26"/>
-      <c r="D32" s="38"/>
-      <c r="E32" s="39"/>
+      <c r="D32" s="39"/>
+      <c r="E32" s="40"/>
     </row>
     <row r="33" spans="1:5" ht="14.4">
-      <c r="A33" s="38"/>
-      <c r="B33" s="39"/>
+      <c r="A33" s="39"/>
+      <c r="B33" s="40"/>
       <c r="C33" s="26"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="39"/>
+      <c r="D33" s="39"/>
+      <c r="E33" s="40"/>
     </row>
     <row r="34" spans="1:5" ht="14.4">
-      <c r="A34" s="38"/>
-      <c r="B34" s="39"/>
+      <c r="A34" s="39"/>
+      <c r="B34" s="40"/>
       <c r="C34" s="26"/>
-      <c r="D34" s="38"/>
-      <c r="E34" s="39"/>
+      <c r="D34" s="39"/>
+      <c r="E34" s="40"/>
     </row>
     <row r="35" spans="1:5" ht="14.4">
-      <c r="A35" s="38"/>
-      <c r="B35" s="39"/>
+      <c r="A35" s="39"/>
+      <c r="B35" s="40"/>
       <c r="C35" s="26"/>
-      <c r="D35" s="38"/>
-      <c r="E35" s="39"/>
+      <c r="D35" s="39"/>
+      <c r="E35" s="40"/>
     </row>
     <row r="36" spans="1:5" ht="14.4">
-      <c r="A36" s="38"/>
-      <c r="B36" s="39"/>
+      <c r="A36" s="39"/>
+      <c r="B36" s="40"/>
       <c r="C36" s="26"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="39"/>
+      <c r="D36" s="39"/>
+      <c r="E36" s="40"/>
     </row>
     <row r="37" spans="1:5" ht="14.4">
-      <c r="A37" s="40"/>
-      <c r="B37" s="41"/>
+      <c r="A37" s="41"/>
+      <c r="B37" s="42"/>
       <c r="C37" s="26"/>
-      <c r="D37" s="40"/>
-      <c r="E37" s="41"/>
+      <c r="D37" s="41"/>
+      <c r="E37" s="42"/>
     </row>
     <row r="38" spans="1:5" ht="14.4">
       <c r="A38" s="26"/>
@@ -2949,253 +2995,257 @@
       <c r="E38" s="26"/>
     </row>
     <row r="39" spans="1:5" ht="17.399999999999999">
-      <c r="A39" s="35" t="s">
+      <c r="A39" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="B39" s="34"/>
+      <c r="B39" s="28"/>
       <c r="C39" s="26"/>
-      <c r="D39" s="35" t="s">
+      <c r="D39" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="E39" s="34"/>
+      <c r="E39" s="28"/>
     </row>
     <row r="40" spans="1:5" ht="14.4">
-      <c r="A40" s="36"/>
-      <c r="B40" s="37"/>
+      <c r="A40" s="37" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+      <c r="B40" s="38"/>
       <c r="C40" s="26"/>
-      <c r="D40" s="36"/>
-      <c r="E40" s="37"/>
+      <c r="D40" s="37" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E40" s="38"/>
     </row>
     <row r="41" spans="1:5" ht="14.4">
-      <c r="A41" s="38"/>
-      <c r="B41" s="39"/>
+      <c r="A41" s="39"/>
+      <c r="B41" s="40"/>
       <c r="C41" s="26"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="39"/>
+      <c r="D41" s="39"/>
+      <c r="E41" s="40"/>
     </row>
     <row r="42" spans="1:5" ht="14.4">
-      <c r="A42" s="38"/>
-      <c r="B42" s="39"/>
+      <c r="A42" s="39"/>
+      <c r="B42" s="40"/>
       <c r="C42" s="26"/>
-      <c r="D42" s="38"/>
-      <c r="E42" s="39"/>
+      <c r="D42" s="39"/>
+      <c r="E42" s="40"/>
     </row>
     <row r="43" spans="1:5" ht="14.4">
-      <c r="A43" s="38"/>
-      <c r="B43" s="39"/>
+      <c r="A43" s="39"/>
+      <c r="B43" s="40"/>
       <c r="C43" s="26"/>
-      <c r="D43" s="38"/>
-      <c r="E43" s="39"/>
+      <c r="D43" s="39"/>
+      <c r="E43" s="40"/>
     </row>
     <row r="44" spans="1:5" ht="14.4">
-      <c r="A44" s="38"/>
-      <c r="B44" s="39"/>
+      <c r="A44" s="39"/>
+      <c r="B44" s="40"/>
       <c r="C44" s="26"/>
-      <c r="D44" s="38"/>
-      <c r="E44" s="39"/>
+      <c r="D44" s="39"/>
+      <c r="E44" s="40"/>
     </row>
     <row r="45" spans="1:5" ht="14.4">
-      <c r="A45" s="38"/>
-      <c r="B45" s="39"/>
+      <c r="A45" s="39"/>
+      <c r="B45" s="40"/>
       <c r="C45" s="26"/>
-      <c r="D45" s="38"/>
-      <c r="E45" s="39"/>
+      <c r="D45" s="39"/>
+      <c r="E45" s="40"/>
     </row>
     <row r="46" spans="1:5" ht="14.4">
-      <c r="A46" s="38"/>
-      <c r="B46" s="39"/>
+      <c r="A46" s="39"/>
+      <c r="B46" s="40"/>
       <c r="C46" s="26"/>
-      <c r="D46" s="38"/>
-      <c r="E46" s="39"/>
+      <c r="D46" s="39"/>
+      <c r="E46" s="40"/>
     </row>
     <row r="47" spans="1:5" ht="14.4">
-      <c r="A47" s="38"/>
-      <c r="B47" s="39"/>
+      <c r="A47" s="39"/>
+      <c r="B47" s="40"/>
       <c r="C47" s="26"/>
-      <c r="D47" s="38"/>
-      <c r="E47" s="39"/>
+      <c r="D47" s="39"/>
+      <c r="E47" s="40"/>
     </row>
     <row r="48" spans="1:5" ht="14.4">
-      <c r="A48" s="38"/>
-      <c r="B48" s="39"/>
+      <c r="A48" s="39"/>
+      <c r="B48" s="40"/>
       <c r="C48" s="26"/>
-      <c r="D48" s="38"/>
-      <c r="E48" s="39"/>
+      <c r="D48" s="39"/>
+      <c r="E48" s="40"/>
     </row>
     <row r="49" spans="1:5" ht="14.4">
-      <c r="A49" s="38"/>
-      <c r="B49" s="39"/>
+      <c r="A49" s="39"/>
+      <c r="B49" s="40"/>
       <c r="C49" s="26"/>
-      <c r="D49" s="38"/>
-      <c r="E49" s="39"/>
+      <c r="D49" s="39"/>
+      <c r="E49" s="40"/>
     </row>
     <row r="50" spans="1:5" ht="14.4">
-      <c r="A50" s="38"/>
-      <c r="B50" s="39"/>
+      <c r="A50" s="39"/>
+      <c r="B50" s="40"/>
       <c r="C50" s="26"/>
-      <c r="D50" s="38"/>
-      <c r="E50" s="39"/>
+      <c r="D50" s="39"/>
+      <c r="E50" s="40"/>
     </row>
     <row r="51" spans="1:5" ht="14.4">
-      <c r="A51" s="38"/>
-      <c r="B51" s="39"/>
+      <c r="A51" s="39"/>
+      <c r="B51" s="40"/>
       <c r="C51" s="26"/>
-      <c r="D51" s="38"/>
-      <c r="E51" s="39"/>
+      <c r="D51" s="39"/>
+      <c r="E51" s="40"/>
     </row>
     <row r="52" spans="1:5" ht="14.4">
-      <c r="A52" s="38"/>
-      <c r="B52" s="39"/>
+      <c r="A52" s="39"/>
+      <c r="B52" s="40"/>
       <c r="C52" s="26"/>
-      <c r="D52" s="38"/>
-      <c r="E52" s="39"/>
+      <c r="D52" s="39"/>
+      <c r="E52" s="40"/>
     </row>
     <row r="53" spans="1:5" ht="14.4">
-      <c r="A53" s="38"/>
-      <c r="B53" s="39"/>
+      <c r="A53" s="39"/>
+      <c r="B53" s="40"/>
       <c r="C53" s="26"/>
-      <c r="D53" s="38"/>
-      <c r="E53" s="39"/>
+      <c r="D53" s="39"/>
+      <c r="E53" s="40"/>
     </row>
     <row r="54" spans="1:5" ht="14.4">
-      <c r="A54" s="38"/>
-      <c r="B54" s="39"/>
+      <c r="A54" s="39"/>
+      <c r="B54" s="40"/>
       <c r="C54" s="26"/>
-      <c r="D54" s="38"/>
-      <c r="E54" s="39"/>
+      <c r="D54" s="39"/>
+      <c r="E54" s="40"/>
     </row>
     <row r="55" spans="1:5" ht="14.4">
-      <c r="A55" s="38"/>
-      <c r="B55" s="39"/>
+      <c r="A55" s="39"/>
+      <c r="B55" s="40"/>
       <c r="C55" s="26"/>
-      <c r="D55" s="38"/>
-      <c r="E55" s="39"/>
+      <c r="D55" s="39"/>
+      <c r="E55" s="40"/>
     </row>
     <row r="56" spans="1:5" ht="14.4">
-      <c r="A56" s="38"/>
-      <c r="B56" s="39"/>
+      <c r="A56" s="39"/>
+      <c r="B56" s="40"/>
       <c r="C56" s="26"/>
-      <c r="D56" s="38"/>
-      <c r="E56" s="39"/>
+      <c r="D56" s="39"/>
+      <c r="E56" s="40"/>
     </row>
     <row r="57" spans="1:5" ht="14.4">
-      <c r="A57" s="38"/>
-      <c r="B57" s="39"/>
+      <c r="A57" s="39"/>
+      <c r="B57" s="40"/>
       <c r="C57" s="26"/>
-      <c r="D57" s="38"/>
-      <c r="E57" s="39"/>
+      <c r="D57" s="39"/>
+      <c r="E57" s="40"/>
     </row>
     <row r="58" spans="1:5" ht="14.4">
-      <c r="A58" s="38"/>
-      <c r="B58" s="39"/>
+      <c r="A58" s="39"/>
+      <c r="B58" s="40"/>
       <c r="C58" s="26"/>
-      <c r="D58" s="38"/>
-      <c r="E58" s="39"/>
+      <c r="D58" s="39"/>
+      <c r="E58" s="40"/>
     </row>
     <row r="59" spans="1:5" ht="14.4">
-      <c r="A59" s="38"/>
-      <c r="B59" s="39"/>
+      <c r="A59" s="39"/>
+      <c r="B59" s="40"/>
       <c r="C59" s="26"/>
-      <c r="D59" s="38"/>
-      <c r="E59" s="39"/>
+      <c r="D59" s="39"/>
+      <c r="E59" s="40"/>
     </row>
     <row r="60" spans="1:5" ht="14.4">
-      <c r="A60" s="38"/>
-      <c r="B60" s="39"/>
+      <c r="A60" s="39"/>
+      <c r="B60" s="40"/>
       <c r="C60" s="26"/>
-      <c r="D60" s="38"/>
-      <c r="E60" s="39"/>
+      <c r="D60" s="39"/>
+      <c r="E60" s="40"/>
     </row>
     <row r="61" spans="1:5" ht="14.4">
-      <c r="A61" s="38"/>
-      <c r="B61" s="39"/>
+      <c r="A61" s="39"/>
+      <c r="B61" s="40"/>
       <c r="C61" s="26"/>
-      <c r="D61" s="38"/>
-      <c r="E61" s="39"/>
+      <c r="D61" s="39"/>
+      <c r="E61" s="40"/>
     </row>
     <row r="62" spans="1:5" ht="14.4">
-      <c r="A62" s="38"/>
-      <c r="B62" s="39"/>
+      <c r="A62" s="39"/>
+      <c r="B62" s="40"/>
       <c r="C62" s="26"/>
-      <c r="D62" s="38"/>
-      <c r="E62" s="39"/>
+      <c r="D62" s="39"/>
+      <c r="E62" s="40"/>
     </row>
     <row r="63" spans="1:5" ht="14.4">
-      <c r="A63" s="38"/>
-      <c r="B63" s="39"/>
+      <c r="A63" s="39"/>
+      <c r="B63" s="40"/>
       <c r="C63" s="26"/>
-      <c r="D63" s="38"/>
-      <c r="E63" s="39"/>
+      <c r="D63" s="39"/>
+      <c r="E63" s="40"/>
     </row>
     <row r="64" spans="1:5" ht="14.4">
-      <c r="A64" s="38"/>
-      <c r="B64" s="39"/>
+      <c r="A64" s="39"/>
+      <c r="B64" s="40"/>
       <c r="C64" s="26"/>
-      <c r="D64" s="38"/>
-      <c r="E64" s="39"/>
+      <c r="D64" s="39"/>
+      <c r="E64" s="40"/>
     </row>
     <row r="65" spans="1:5" ht="14.4">
-      <c r="A65" s="38"/>
-      <c r="B65" s="39"/>
+      <c r="A65" s="39"/>
+      <c r="B65" s="40"/>
       <c r="C65" s="26"/>
-      <c r="D65" s="38"/>
-      <c r="E65" s="39"/>
+      <c r="D65" s="39"/>
+      <c r="E65" s="40"/>
     </row>
     <row r="66" spans="1:5" ht="14.4">
-      <c r="A66" s="38"/>
-      <c r="B66" s="39"/>
+      <c r="A66" s="39"/>
+      <c r="B66" s="40"/>
       <c r="C66" s="26"/>
-      <c r="D66" s="38"/>
-      <c r="E66" s="39"/>
+      <c r="D66" s="39"/>
+      <c r="E66" s="40"/>
     </row>
     <row r="67" spans="1:5" ht="14.4">
-      <c r="A67" s="38"/>
-      <c r="B67" s="39"/>
+      <c r="A67" s="39"/>
+      <c r="B67" s="40"/>
       <c r="C67" s="26"/>
-      <c r="D67" s="38"/>
-      <c r="E67" s="39"/>
+      <c r="D67" s="39"/>
+      <c r="E67" s="40"/>
     </row>
     <row r="68" spans="1:5" ht="14.4">
-      <c r="A68" s="38"/>
-      <c r="B68" s="39"/>
+      <c r="A68" s="39"/>
+      <c r="B68" s="40"/>
       <c r="C68" s="26"/>
-      <c r="D68" s="38"/>
-      <c r="E68" s="39"/>
+      <c r="D68" s="39"/>
+      <c r="E68" s="40"/>
     </row>
     <row r="69" spans="1:5" ht="14.4">
-      <c r="A69" s="38"/>
-      <c r="B69" s="39"/>
+      <c r="A69" s="39"/>
+      <c r="B69" s="40"/>
       <c r="C69" s="26"/>
-      <c r="D69" s="38"/>
-      <c r="E69" s="39"/>
+      <c r="D69" s="39"/>
+      <c r="E69" s="40"/>
     </row>
     <row r="70" spans="1:5" ht="14.4">
-      <c r="A70" s="38"/>
-      <c r="B70" s="39"/>
+      <c r="A70" s="39"/>
+      <c r="B70" s="40"/>
       <c r="C70" s="26"/>
-      <c r="D70" s="38"/>
-      <c r="E70" s="39"/>
+      <c r="D70" s="39"/>
+      <c r="E70" s="40"/>
     </row>
     <row r="71" spans="1:5" ht="14.4">
-      <c r="A71" s="38"/>
-      <c r="B71" s="39"/>
+      <c r="A71" s="39"/>
+      <c r="B71" s="40"/>
       <c r="C71" s="26"/>
-      <c r="D71" s="38"/>
-      <c r="E71" s="39"/>
+      <c r="D71" s="39"/>
+      <c r="E71" s="40"/>
     </row>
     <row r="72" spans="1:5" ht="14.4">
-      <c r="A72" s="38"/>
-      <c r="B72" s="39"/>
+      <c r="A72" s="39"/>
+      <c r="B72" s="40"/>
       <c r="C72" s="26"/>
-      <c r="D72" s="38"/>
-      <c r="E72" s="39"/>
+      <c r="D72" s="39"/>
+      <c r="E72" s="40"/>
     </row>
     <row r="73" spans="1:5" ht="14.4">
-      <c r="A73" s="40"/>
-      <c r="B73" s="41"/>
+      <c r="A73" s="41"/>
+      <c r="B73" s="42"/>
       <c r="C73" s="26"/>
-      <c r="D73" s="40"/>
-      <c r="E73" s="41"/>
+      <c r="D73" s="41"/>
+      <c r="E73" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -3210,6 +3260,5 @@
     <mergeCell ref="A40:B73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>